<commit_message>
Add unique daily borrowers and set zoom on all files
</commit_message>
<xml_diff>
--- a/statistics_files/2026/2026_99_a_cy_monthly_overview.xlsx
+++ b/statistics_files/2026/2026_99_a_cy_monthly_overview.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\George\Documents\github\next_statistics\statistics_files\2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C58452F4-74FA-40C5-82BA-426B335B8156}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2230CB8-6269-46F2-8D1A-4486D8918861}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="872" xr2:uid="{6DE01D01-D2C0-4362-AEEE-36DB0900D2F9}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="872" xr2:uid="{6DE01D01-D2C0-4362-AEEE-36DB0900D2F9}"/>
   </bookViews>
   <sheets>
     <sheet name="Year total" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Standardize all files for 2026
</commit_message>
<xml_diff>
--- a/statistics_files/2026/2026_99_a_cy_monthly_overview.xlsx
+++ b/statistics_files/2026/2026_99_a_cy_monthly_overview.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\George\Documents\github\next_statistics\statistics_files\2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2230CB8-6269-46F2-8D1A-4486D8918861}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{787E0274-08C3-450E-8CD5-54D894435E59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="872" xr2:uid="{6DE01D01-D2C0-4362-AEEE-36DB0900D2F9}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="872" xr2:uid="{6DE01D01-D2C0-4362-AEEE-36DB0900D2F9}"/>
   </bookViews>
   <sheets>
-    <sheet name="Year total" sheetId="1" r:id="rId1"/>
+    <sheet name="Yearly total" sheetId="1" r:id="rId1"/>
     <sheet name="Items added summary" sheetId="14" r:id="rId2"/>
     <sheet name="Items deleted summary" sheetId="15" r:id="rId3"/>
     <sheet name="January" sheetId="2" r:id="rId4"/>
@@ -59,7 +59,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="23" hidden="1">November!$A$1:$U$57</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="21" hidden="1">October!$A$1:$U$57</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">September!$A$1:$U$57</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Year total'!$A$1:$V$57</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Yearly total'!$A$1:$V$57</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35018,7 +35018,7 @@
         <v>21</v>
       </c>
       <c r="B2" s="35">
-        <f>'Year total'!B2</f>
+        <f>'Yearly total'!B2</f>
         <v>62728</v>
       </c>
       <c r="C2" s="52">
@@ -35095,7 +35095,7 @@
         <v>22</v>
       </c>
       <c r="B3" s="37">
-        <f>'Year total'!B3</f>
+        <f>'Yearly total'!B3</f>
         <v>26955</v>
       </c>
       <c r="C3" s="53">
@@ -35172,7 +35172,7 @@
         <v>23</v>
       </c>
       <c r="B4" s="35">
-        <f>'Year total'!B4</f>
+        <f>'Yearly total'!B4</f>
         <v>61759</v>
       </c>
       <c r="C4" s="52">
@@ -35249,7 +35249,7 @@
         <v>24</v>
       </c>
       <c r="B5" s="37">
-        <f>'Year total'!B5</f>
+        <f>'Yearly total'!B5</f>
         <v>12931</v>
       </c>
       <c r="C5" s="53">
@@ -35326,7 +35326,7 @@
         <v>25</v>
       </c>
       <c r="B6" s="35">
-        <f>'Year total'!B6</f>
+        <f>'Yearly total'!B6</f>
         <v>62279</v>
       </c>
       <c r="C6" s="52">
@@ -35403,7 +35403,7 @@
         <v>26</v>
       </c>
       <c r="B7" s="37">
-        <f>'Year total'!B7</f>
+        <f>'Yearly total'!B7</f>
         <v>14098</v>
       </c>
       <c r="C7" s="53">
@@ -35480,7 +35480,7 @@
         <v>27</v>
       </c>
       <c r="B8" s="35">
-        <f>'Year total'!B8</f>
+        <f>'Yearly total'!B8</f>
         <v>7220</v>
       </c>
       <c r="C8" s="52">
@@ -35557,7 +35557,7 @@
         <v>28</v>
       </c>
       <c r="B9" s="37">
-        <f>'Year total'!B9</f>
+        <f>'Yearly total'!B9</f>
         <v>8932</v>
       </c>
       <c r="C9" s="53">
@@ -35634,7 +35634,7 @@
         <v>29</v>
       </c>
       <c r="B10" s="35">
-        <f>'Year total'!B10</f>
+        <f>'Yearly total'!B10</f>
         <v>6339</v>
       </c>
       <c r="C10" s="52">
@@ -35711,7 +35711,7 @@
         <v>30</v>
       </c>
       <c r="B11" s="37">
-        <f>'Year total'!B11</f>
+        <f>'Yearly total'!B11</f>
         <v>365</v>
       </c>
       <c r="C11" s="53">
@@ -35788,7 +35788,7 @@
         <v>31</v>
       </c>
       <c r="B12" s="39">
-        <f>'Year total'!B12</f>
+        <f>'Yearly total'!B12</f>
         <v>2135</v>
       </c>
       <c r="C12" s="54">
@@ -35865,7 +35865,7 @@
         <v>32</v>
       </c>
       <c r="B13" s="41">
-        <f>'Year total'!B13</f>
+        <f>'Yearly total'!B13</f>
         <v>5236</v>
       </c>
       <c r="C13" s="55">
@@ -35942,7 +35942,7 @@
         <v>33</v>
       </c>
       <c r="B14" s="39">
-        <f>'Year total'!B14</f>
+        <f>'Yearly total'!B14</f>
         <v>11712</v>
       </c>
       <c r="C14" s="54">
@@ -36019,7 +36019,7 @@
         <v>34</v>
       </c>
       <c r="B15" s="41">
-        <f>'Year total'!B15</f>
+        <f>'Yearly total'!B15</f>
         <v>8517</v>
       </c>
       <c r="C15" s="55">
@@ -36096,7 +36096,7 @@
         <v>35</v>
       </c>
       <c r="B16" s="35">
-        <f>'Year total'!B16</f>
+        <f>'Yearly total'!B16</f>
         <v>8430</v>
       </c>
       <c r="C16" s="52">
@@ -36173,7 +36173,7 @@
         <v>36</v>
       </c>
       <c r="B17" s="37">
-        <f>'Year total'!B17</f>
+        <f>'Yearly total'!B17</f>
         <v>14088</v>
       </c>
       <c r="C17" s="53">
@@ -36250,7 +36250,7 @@
         <v>37</v>
       </c>
       <c r="B18" s="35">
-        <f>'Year total'!B18</f>
+        <f>'Yearly total'!B18</f>
         <v>7390</v>
       </c>
       <c r="C18" s="52">
@@ -36327,7 +36327,7 @@
         <v>38</v>
       </c>
       <c r="B19" s="37">
-        <f>'Year total'!B19</f>
+        <f>'Yearly total'!B19</f>
         <v>32250</v>
       </c>
       <c r="C19" s="53">
@@ -36404,7 +36404,7 @@
         <v>39</v>
       </c>
       <c r="B20" s="35">
-        <f>'Year total'!B20</f>
+        <f>'Yearly total'!B20</f>
         <v>2688</v>
       </c>
       <c r="C20" s="52">
@@ -36481,7 +36481,7 @@
         <v>40</v>
       </c>
       <c r="B21" s="37">
-        <f>'Year total'!B21</f>
+        <f>'Yearly total'!B21</f>
         <v>26563</v>
       </c>
       <c r="C21" s="53">
@@ -36558,7 +36558,7 @@
         <v>41</v>
       </c>
       <c r="B22" s="35">
-        <f>'Year total'!B22</f>
+        <f>'Yearly total'!B22</f>
         <v>13769</v>
       </c>
       <c r="C22" s="52">
@@ -36635,7 +36635,7 @@
         <v>42</v>
       </c>
       <c r="B23" s="37">
-        <f>'Year total'!B23</f>
+        <f>'Yearly total'!B23</f>
         <v>24586</v>
       </c>
       <c r="C23" s="53">
@@ -36712,7 +36712,7 @@
         <v>43</v>
       </c>
       <c r="B24" s="35">
-        <f>'Year total'!B24</f>
+        <f>'Yearly total'!B24</f>
         <v>86339</v>
       </c>
       <c r="C24" s="52">
@@ -36789,7 +36789,7 @@
         <v>44</v>
       </c>
       <c r="B25" s="37">
-        <f>'Year total'!B25</f>
+        <f>'Yearly total'!B25</f>
         <v>13058</v>
       </c>
       <c r="C25" s="53">
@@ -36866,7 +36866,7 @@
         <v>45</v>
       </c>
       <c r="B26" s="35">
-        <f>'Year total'!B26</f>
+        <f>'Yearly total'!B26</f>
         <v>0</v>
       </c>
       <c r="C26" s="52">
@@ -36943,7 +36943,7 @@
         <v>46</v>
       </c>
       <c r="B27" s="37">
-        <f>'Year total'!B27</f>
+        <f>'Yearly total'!B27</f>
         <v>11888</v>
       </c>
       <c r="C27" s="53">
@@ -37020,7 +37020,7 @@
         <v>47</v>
       </c>
       <c r="B28" s="35">
-        <f>'Year total'!B28</f>
+        <f>'Yearly total'!B28</f>
         <v>4728</v>
       </c>
       <c r="C28" s="52">
@@ -37097,7 +37097,7 @@
         <v>48</v>
       </c>
       <c r="B29" s="37">
-        <f>'Year total'!B29</f>
+        <f>'Yearly total'!B29</f>
         <v>16243</v>
       </c>
       <c r="C29" s="53">
@@ -37174,7 +37174,7 @@
         <v>49</v>
       </c>
       <c r="B30" s="35">
-        <f>'Year total'!B30</f>
+        <f>'Yearly total'!B30</f>
         <v>948</v>
       </c>
       <c r="C30" s="52">
@@ -37251,7 +37251,7 @@
         <v>50</v>
       </c>
       <c r="B31" s="37">
-        <f>'Year total'!B31</f>
+        <f>'Yearly total'!B31</f>
         <v>15766</v>
       </c>
       <c r="C31" s="53">
@@ -37328,7 +37328,7 @@
         <v>51</v>
       </c>
       <c r="B32" s="35">
-        <f>'Year total'!B32</f>
+        <f>'Yearly total'!B32</f>
         <v>19867</v>
       </c>
       <c r="C32" s="52">
@@ -37405,7 +37405,7 @@
         <v>52</v>
       </c>
       <c r="B33" s="37">
-        <f>'Year total'!B33</f>
+        <f>'Yearly total'!B33</f>
         <v>19677</v>
       </c>
       <c r="C33" s="53">
@@ -37482,7 +37482,7 @@
         <v>53</v>
       </c>
       <c r="B34" s="35">
-        <f>'Year total'!B34</f>
+        <f>'Yearly total'!B34</f>
         <v>10510</v>
       </c>
       <c r="C34" s="52">
@@ -37559,7 +37559,7 @@
         <v>54</v>
       </c>
       <c r="B35" s="37">
-        <f>'Year total'!B35</f>
+        <f>'Yearly total'!B35</f>
         <v>72390</v>
       </c>
       <c r="C35" s="53">
@@ -37636,7 +37636,7 @@
         <v>55</v>
       </c>
       <c r="B36" s="35">
-        <f>'Year total'!B36</f>
+        <f>'Yearly total'!B36</f>
         <v>22348</v>
       </c>
       <c r="C36" s="52">
@@ -37713,7 +37713,7 @@
         <v>56</v>
       </c>
       <c r="B37" s="37">
-        <f>'Year total'!B37</f>
+        <f>'Yearly total'!B37</f>
         <v>26630</v>
       </c>
       <c r="C37" s="53">
@@ -37790,7 +37790,7 @@
         <v>57</v>
       </c>
       <c r="B38" s="35">
-        <f>'Year total'!B38</f>
+        <f>'Yearly total'!B38</f>
         <v>13515</v>
       </c>
       <c r="C38" s="52">
@@ -37867,7 +37867,7 @@
         <v>62</v>
       </c>
       <c r="B39" s="37">
-        <f>'Year total'!B39</f>
+        <f>'Yearly total'!B39</f>
         <v>6769</v>
       </c>
       <c r="C39" s="53">
@@ -37944,7 +37944,7 @@
         <v>58</v>
       </c>
       <c r="B40" s="43">
-        <f>'Year total'!B40</f>
+        <f>'Yearly total'!B40</f>
         <v>10705</v>
       </c>
       <c r="C40" s="56">
@@ -38021,7 +38021,7 @@
         <v>59</v>
       </c>
       <c r="B41" s="45">
-        <f>'Year total'!B41</f>
+        <f>'Yearly total'!B41</f>
         <v>16302</v>
       </c>
       <c r="C41" s="57">
@@ -38098,7 +38098,7 @@
         <v>60</v>
       </c>
       <c r="B42" s="43">
-        <f>'Year total'!B42</f>
+        <f>'Yearly total'!B42</f>
         <v>4103</v>
       </c>
       <c r="C42" s="56">
@@ -38175,7 +38175,7 @@
         <v>61</v>
       </c>
       <c r="B43" s="45">
-        <f>'Year total'!B43</f>
+        <f>'Yearly total'!B43</f>
         <v>4994</v>
       </c>
       <c r="C43" s="57">
@@ -38252,7 +38252,7 @@
         <v>63</v>
       </c>
       <c r="B44" s="37">
-        <f>'Year total'!B44</f>
+        <f>'Yearly total'!B44</f>
         <v>8593</v>
       </c>
       <c r="C44" s="53">
@@ -38329,7 +38329,7 @@
         <v>64</v>
       </c>
       <c r="B45" s="35">
-        <f>'Year total'!B45</f>
+        <f>'Yearly total'!B45</f>
         <v>16392</v>
       </c>
       <c r="C45" s="52">
@@ -38406,7 +38406,7 @@
         <v>65</v>
       </c>
       <c r="B46" s="37">
-        <f>'Year total'!B46</f>
+        <f>'Yearly total'!B46</f>
         <v>29245</v>
       </c>
       <c r="C46" s="53">
@@ -38483,7 +38483,7 @@
         <v>66</v>
       </c>
       <c r="B47" s="35">
-        <f>'Year total'!B47</f>
+        <f>'Yearly total'!B47</f>
         <v>21662</v>
       </c>
       <c r="C47" s="52">
@@ -38560,7 +38560,7 @@
         <v>67</v>
       </c>
       <c r="B48" s="37">
-        <f>'Year total'!B48</f>
+        <f>'Yearly total'!B48</f>
         <v>9839</v>
       </c>
       <c r="C48" s="53">
@@ -38637,7 +38637,7 @@
         <v>68</v>
       </c>
       <c r="B49" s="35">
-        <f>'Year total'!B49</f>
+        <f>'Yearly total'!B49</f>
         <v>26794</v>
       </c>
       <c r="C49" s="52">
@@ -38714,7 +38714,7 @@
         <v>69</v>
       </c>
       <c r="B50" s="37">
-        <f>'Year total'!B50</f>
+        <f>'Yearly total'!B50</f>
         <v>8498</v>
       </c>
       <c r="C50" s="53">
@@ -38791,7 +38791,7 @@
         <v>70</v>
       </c>
       <c r="B51" s="35">
-        <f>'Year total'!B51</f>
+        <f>'Yearly total'!B51</f>
         <v>21537</v>
       </c>
       <c r="C51" s="52">
@@ -38868,7 +38868,7 @@
         <v>71</v>
       </c>
       <c r="B52" s="37">
-        <f>'Year total'!B52</f>
+        <f>'Yearly total'!B52</f>
         <v>10310</v>
       </c>
       <c r="C52" s="53">
@@ -38945,7 +38945,7 @@
         <v>72</v>
       </c>
       <c r="B53" s="35">
-        <f>'Year total'!B53</f>
+        <f>'Yearly total'!B53</f>
         <v>14087</v>
       </c>
       <c r="C53" s="52">
@@ -39022,7 +39022,7 @@
         <v>73</v>
       </c>
       <c r="B54" s="37">
-        <f>'Year total'!B54</f>
+        <f>'Yearly total'!B54</f>
         <v>7577</v>
       </c>
       <c r="C54" s="53">
@@ -39099,7 +39099,7 @@
         <v>93</v>
       </c>
       <c r="B55" s="47">
-        <f>'Year total'!B55</f>
+        <f>'Yearly total'!B55</f>
         <v>27600</v>
       </c>
       <c r="C55" s="58">
@@ -39176,7 +39176,7 @@
         <v>94</v>
       </c>
       <c r="B56" s="49">
-        <f>'Year total'!B56</f>
+        <f>'Yearly total'!B56</f>
         <v>36104</v>
       </c>
       <c r="C56" s="59">
@@ -61067,51 +61067,51 @@
         <v>145</v>
       </c>
       <c r="B8" t="str">
-        <f>CONCATENATE("            &lt;td&gt;",'Year total'!$J$57,"&lt;/td&gt;")</f>
+        <f>CONCATENATE("            &lt;td&gt;",'Yearly total'!$J$57,"&lt;/td&gt;")</f>
         <v xml:space="preserve">            &lt;td&gt;86140&lt;/td&gt;</v>
       </c>
       <c r="C8" t="str">
-        <f>CONCATENATE("            &lt;td&gt;",'Year total'!$J$57,"&lt;/td&gt;")</f>
+        <f>CONCATENATE("            &lt;td&gt;",'Yearly total'!$J$57,"&lt;/td&gt;")</f>
         <v xml:space="preserve">            &lt;td&gt;86140&lt;/td&gt;</v>
       </c>
       <c r="D8" t="str">
-        <f>CONCATENATE("            &lt;td&gt;",'Year total'!$J$57,"&lt;/td&gt;")</f>
+        <f>CONCATENATE("            &lt;td&gt;",'Yearly total'!$J$57,"&lt;/td&gt;")</f>
         <v xml:space="preserve">            &lt;td&gt;86140&lt;/td&gt;</v>
       </c>
       <c r="E8" t="str">
-        <f>CONCATENATE("            &lt;td&gt;",'Year total'!$J$57,"&lt;/td&gt;")</f>
+        <f>CONCATENATE("            &lt;td&gt;",'Yearly total'!$J$57,"&lt;/td&gt;")</f>
         <v xml:space="preserve">            &lt;td&gt;86140&lt;/td&gt;</v>
       </c>
       <c r="F8" t="str">
-        <f>CONCATENATE("            &lt;td&gt;",'Year total'!$J$57,"&lt;/td&gt;")</f>
+        <f>CONCATENATE("            &lt;td&gt;",'Yearly total'!$J$57,"&lt;/td&gt;")</f>
         <v xml:space="preserve">            &lt;td&gt;86140&lt;/td&gt;</v>
       </c>
       <c r="G8" t="str">
-        <f>CONCATENATE("            &lt;td&gt;",'Year total'!$J$57,"&lt;/td&gt;")</f>
+        <f>CONCATENATE("            &lt;td&gt;",'Yearly total'!$J$57,"&lt;/td&gt;")</f>
         <v xml:space="preserve">            &lt;td&gt;86140&lt;/td&gt;</v>
       </c>
       <c r="H8" t="str">
-        <f>CONCATENATE("            &lt;td&gt;",'Year total'!$J$57,"&lt;/td&gt;")</f>
+        <f>CONCATENATE("            &lt;td&gt;",'Yearly total'!$J$57,"&lt;/td&gt;")</f>
         <v xml:space="preserve">            &lt;td&gt;86140&lt;/td&gt;</v>
       </c>
       <c r="I8" t="str">
-        <f>CONCATENATE("            &lt;td&gt;",'Year total'!$J$57,"&lt;/td&gt;")</f>
+        <f>CONCATENATE("            &lt;td&gt;",'Yearly total'!$J$57,"&lt;/td&gt;")</f>
         <v xml:space="preserve">            &lt;td&gt;86140&lt;/td&gt;</v>
       </c>
       <c r="J8" t="str">
-        <f>CONCATENATE("            &lt;td&gt;",'Year total'!$J$57,"&lt;/td&gt;")</f>
+        <f>CONCATENATE("            &lt;td&gt;",'Yearly total'!$J$57,"&lt;/td&gt;")</f>
         <v xml:space="preserve">            &lt;td&gt;86140&lt;/td&gt;</v>
       </c>
       <c r="K8" t="str">
-        <f>CONCATENATE("            &lt;td&gt;",'Year total'!$J$57,"&lt;/td&gt;")</f>
+        <f>CONCATENATE("            &lt;td&gt;",'Yearly total'!$J$57,"&lt;/td&gt;")</f>
         <v xml:space="preserve">            &lt;td&gt;86140&lt;/td&gt;</v>
       </c>
       <c r="L8" t="str">
-        <f>CONCATENATE("            &lt;td&gt;",'Year total'!$J$57,"&lt;/td&gt;")</f>
+        <f>CONCATENATE("            &lt;td&gt;",'Yearly total'!$J$57,"&lt;/td&gt;")</f>
         <v xml:space="preserve">            &lt;td&gt;86140&lt;/td&gt;</v>
       </c>
       <c r="M8" t="str">
-        <f>CONCATENATE("            &lt;td&gt;",'Year total'!$J$57,"&lt;/td&gt;")</f>
+        <f>CONCATENATE("            &lt;td&gt;",'Yearly total'!$J$57,"&lt;/td&gt;")</f>
         <v xml:space="preserve">            &lt;td&gt;86140&lt;/td&gt;</v>
       </c>
     </row>
@@ -61236,7 +61236,7 @@
         <v>21</v>
       </c>
       <c r="B2" s="5">
-        <f>'Year total'!B2</f>
+        <f>'Yearly total'!B2</f>
         <v>62728</v>
       </c>
       <c r="C2" s="17">
@@ -61313,7 +61313,7 @@
         <v>22</v>
       </c>
       <c r="B3" s="6">
-        <f>'Year total'!B3</f>
+        <f>'Yearly total'!B3</f>
         <v>26955</v>
       </c>
       <c r="C3" s="18">
@@ -61390,7 +61390,7 @@
         <v>23</v>
       </c>
       <c r="B4" s="5">
-        <f>'Year total'!B4</f>
+        <f>'Yearly total'!B4</f>
         <v>61759</v>
       </c>
       <c r="C4" s="17">
@@ -61467,7 +61467,7 @@
         <v>24</v>
       </c>
       <c r="B5" s="6">
-        <f>'Year total'!B5</f>
+        <f>'Yearly total'!B5</f>
         <v>12931</v>
       </c>
       <c r="C5" s="18">
@@ -61544,7 +61544,7 @@
         <v>25</v>
       </c>
       <c r="B6" s="5">
-        <f>'Year total'!B6</f>
+        <f>'Yearly total'!B6</f>
         <v>62279</v>
       </c>
       <c r="C6" s="17">
@@ -61621,7 +61621,7 @@
         <v>26</v>
       </c>
       <c r="B7" s="6">
-        <f>'Year total'!B7</f>
+        <f>'Yearly total'!B7</f>
         <v>14098</v>
       </c>
       <c r="C7" s="18">
@@ -61698,7 +61698,7 @@
         <v>27</v>
       </c>
       <c r="B8" s="5">
-        <f>'Year total'!B8</f>
+        <f>'Yearly total'!B8</f>
         <v>7220</v>
       </c>
       <c r="C8" s="17">
@@ -61775,7 +61775,7 @@
         <v>28</v>
       </c>
       <c r="B9" s="6">
-        <f>'Year total'!B9</f>
+        <f>'Yearly total'!B9</f>
         <v>8932</v>
       </c>
       <c r="C9" s="18">
@@ -61852,7 +61852,7 @@
         <v>29</v>
       </c>
       <c r="B10" s="5">
-        <f>'Year total'!B10</f>
+        <f>'Yearly total'!B10</f>
         <v>6339</v>
       </c>
       <c r="C10" s="17">
@@ -61929,7 +61929,7 @@
         <v>30</v>
       </c>
       <c r="B11" s="6">
-        <f>'Year total'!B11</f>
+        <f>'Yearly total'!B11</f>
         <v>365</v>
       </c>
       <c r="C11" s="18">
@@ -62006,7 +62006,7 @@
         <v>31</v>
       </c>
       <c r="B12" s="7">
-        <f>'Year total'!B12</f>
+        <f>'Yearly total'!B12</f>
         <v>2135</v>
       </c>
       <c r="C12" s="19">
@@ -62083,7 +62083,7 @@
         <v>32</v>
       </c>
       <c r="B13" s="8">
-        <f>'Year total'!B13</f>
+        <f>'Yearly total'!B13</f>
         <v>5236</v>
       </c>
       <c r="C13" s="20">
@@ -62160,7 +62160,7 @@
         <v>33</v>
       </c>
       <c r="B14" s="7">
-        <f>'Year total'!B14</f>
+        <f>'Yearly total'!B14</f>
         <v>11712</v>
       </c>
       <c r="C14" s="19">
@@ -62237,7 +62237,7 @@
         <v>34</v>
       </c>
       <c r="B15" s="8">
-        <f>'Year total'!B15</f>
+        <f>'Yearly total'!B15</f>
         <v>8517</v>
       </c>
       <c r="C15" s="20">
@@ -62314,7 +62314,7 @@
         <v>35</v>
       </c>
       <c r="B16" s="5">
-        <f>'Year total'!B16</f>
+        <f>'Yearly total'!B16</f>
         <v>8430</v>
       </c>
       <c r="C16" s="17">
@@ -62391,7 +62391,7 @@
         <v>36</v>
       </c>
       <c r="B17" s="6">
-        <f>'Year total'!B17</f>
+        <f>'Yearly total'!B17</f>
         <v>14088</v>
       </c>
       <c r="C17" s="18">
@@ -62468,7 +62468,7 @@
         <v>37</v>
       </c>
       <c r="B18" s="5">
-        <f>'Year total'!B18</f>
+        <f>'Yearly total'!B18</f>
         <v>7390</v>
       </c>
       <c r="C18" s="17">
@@ -62545,7 +62545,7 @@
         <v>38</v>
       </c>
       <c r="B19" s="6">
-        <f>'Year total'!B19</f>
+        <f>'Yearly total'!B19</f>
         <v>32250</v>
       </c>
       <c r="C19" s="18">
@@ -62622,7 +62622,7 @@
         <v>39</v>
       </c>
       <c r="B20" s="5">
-        <f>'Year total'!B20</f>
+        <f>'Yearly total'!B20</f>
         <v>2688</v>
       </c>
       <c r="C20" s="17">
@@ -62699,7 +62699,7 @@
         <v>40</v>
       </c>
       <c r="B21" s="6">
-        <f>'Year total'!B21</f>
+        <f>'Yearly total'!B21</f>
         <v>26563</v>
       </c>
       <c r="C21" s="18">
@@ -62776,7 +62776,7 @@
         <v>41</v>
       </c>
       <c r="B22" s="5">
-        <f>'Year total'!B22</f>
+        <f>'Yearly total'!B22</f>
         <v>13769</v>
       </c>
       <c r="C22" s="17">
@@ -62853,7 +62853,7 @@
         <v>42</v>
       </c>
       <c r="B23" s="6">
-        <f>'Year total'!B23</f>
+        <f>'Yearly total'!B23</f>
         <v>24586</v>
       </c>
       <c r="C23" s="18">
@@ -62930,7 +62930,7 @@
         <v>43</v>
       </c>
       <c r="B24" s="5">
-        <f>'Year total'!B24</f>
+        <f>'Yearly total'!B24</f>
         <v>86339</v>
       </c>
       <c r="C24" s="17">
@@ -63007,7 +63007,7 @@
         <v>44</v>
       </c>
       <c r="B25" s="6">
-        <f>'Year total'!B25</f>
+        <f>'Yearly total'!B25</f>
         <v>13058</v>
       </c>
       <c r="C25" s="18">
@@ -63084,7 +63084,7 @@
         <v>45</v>
       </c>
       <c r="B26" s="5">
-        <f>'Year total'!B26</f>
+        <f>'Yearly total'!B26</f>
         <v>0</v>
       </c>
       <c r="C26" s="17">
@@ -63161,7 +63161,7 @@
         <v>46</v>
       </c>
       <c r="B27" s="6">
-        <f>'Year total'!B27</f>
+        <f>'Yearly total'!B27</f>
         <v>11888</v>
       </c>
       <c r="C27" s="18">
@@ -63238,7 +63238,7 @@
         <v>47</v>
       </c>
       <c r="B28" s="5">
-        <f>'Year total'!B28</f>
+        <f>'Yearly total'!B28</f>
         <v>4728</v>
       </c>
       <c r="C28" s="17">
@@ -63315,7 +63315,7 @@
         <v>48</v>
       </c>
       <c r="B29" s="6">
-        <f>'Year total'!B29</f>
+        <f>'Yearly total'!B29</f>
         <v>16243</v>
       </c>
       <c r="C29" s="18">
@@ -63392,7 +63392,7 @@
         <v>49</v>
       </c>
       <c r="B30" s="5">
-        <f>'Year total'!B30</f>
+        <f>'Yearly total'!B30</f>
         <v>948</v>
       </c>
       <c r="C30" s="17">
@@ -63469,7 +63469,7 @@
         <v>50</v>
       </c>
       <c r="B31" s="6">
-        <f>'Year total'!B31</f>
+        <f>'Yearly total'!B31</f>
         <v>15766</v>
       </c>
       <c r="C31" s="18">
@@ -63546,7 +63546,7 @@
         <v>51</v>
       </c>
       <c r="B32" s="5">
-        <f>'Year total'!B32</f>
+        <f>'Yearly total'!B32</f>
         <v>19867</v>
       </c>
       <c r="C32" s="17">
@@ -63623,7 +63623,7 @@
         <v>52</v>
       </c>
       <c r="B33" s="6">
-        <f>'Year total'!B33</f>
+        <f>'Yearly total'!B33</f>
         <v>19677</v>
       </c>
       <c r="C33" s="18">
@@ -63700,7 +63700,7 @@
         <v>53</v>
       </c>
       <c r="B34" s="5">
-        <f>'Year total'!B34</f>
+        <f>'Yearly total'!B34</f>
         <v>10510</v>
       </c>
       <c r="C34" s="17">
@@ -63777,7 +63777,7 @@
         <v>54</v>
       </c>
       <c r="B35" s="6">
-        <f>'Year total'!B35</f>
+        <f>'Yearly total'!B35</f>
         <v>72390</v>
       </c>
       <c r="C35" s="18">
@@ -63854,7 +63854,7 @@
         <v>55</v>
       </c>
       <c r="B36" s="5">
-        <f>'Year total'!B36</f>
+        <f>'Yearly total'!B36</f>
         <v>22348</v>
       </c>
       <c r="C36" s="17">
@@ -63931,7 +63931,7 @@
         <v>56</v>
       </c>
       <c r="B37" s="6">
-        <f>'Year total'!B37</f>
+        <f>'Yearly total'!B37</f>
         <v>26630</v>
       </c>
       <c r="C37" s="18">
@@ -64008,7 +64008,7 @@
         <v>57</v>
       </c>
       <c r="B38" s="5">
-        <f>'Year total'!B38</f>
+        <f>'Yearly total'!B38</f>
         <v>13515</v>
       </c>
       <c r="C38" s="17">
@@ -64085,7 +64085,7 @@
         <v>62</v>
       </c>
       <c r="B39" s="6">
-        <f>'Year total'!B39</f>
+        <f>'Yearly total'!B39</f>
         <v>6769</v>
       </c>
       <c r="C39" s="18">
@@ -64162,7 +64162,7 @@
         <v>58</v>
       </c>
       <c r="B40" s="10">
-        <f>'Year total'!B40</f>
+        <f>'Yearly total'!B40</f>
         <v>10705</v>
       </c>
       <c r="C40" s="21">
@@ -64239,7 +64239,7 @@
         <v>59</v>
       </c>
       <c r="B41" s="9">
-        <f>'Year total'!B41</f>
+        <f>'Yearly total'!B41</f>
         <v>16302</v>
       </c>
       <c r="C41" s="22">
@@ -64316,7 +64316,7 @@
         <v>60</v>
       </c>
       <c r="B42" s="10">
-        <f>'Year total'!B42</f>
+        <f>'Yearly total'!B42</f>
         <v>4103</v>
       </c>
       <c r="C42" s="21">
@@ -64393,7 +64393,7 @@
         <v>61</v>
       </c>
       <c r="B43" s="9">
-        <f>'Year total'!B43</f>
+        <f>'Yearly total'!B43</f>
         <v>4994</v>
       </c>
       <c r="C43" s="22">
@@ -64470,7 +64470,7 @@
         <v>63</v>
       </c>
       <c r="B44" s="6">
-        <f>'Year total'!B44</f>
+        <f>'Yearly total'!B44</f>
         <v>8593</v>
       </c>
       <c r="C44" s="18">
@@ -64547,7 +64547,7 @@
         <v>64</v>
       </c>
       <c r="B45" s="5">
-        <f>'Year total'!B45</f>
+        <f>'Yearly total'!B45</f>
         <v>16392</v>
       </c>
       <c r="C45" s="17">
@@ -64624,7 +64624,7 @@
         <v>65</v>
       </c>
       <c r="B46" s="6">
-        <f>'Year total'!B46</f>
+        <f>'Yearly total'!B46</f>
         <v>29245</v>
       </c>
       <c r="C46" s="18">
@@ -64701,7 +64701,7 @@
         <v>66</v>
       </c>
       <c r="B47" s="5">
-        <f>'Year total'!B47</f>
+        <f>'Yearly total'!B47</f>
         <v>21662</v>
       </c>
       <c r="C47" s="17">
@@ -64778,7 +64778,7 @@
         <v>67</v>
       </c>
       <c r="B48" s="6">
-        <f>'Year total'!B48</f>
+        <f>'Yearly total'!B48</f>
         <v>9839</v>
       </c>
       <c r="C48" s="18">
@@ -64855,7 +64855,7 @@
         <v>68</v>
       </c>
       <c r="B49" s="5">
-        <f>'Year total'!B49</f>
+        <f>'Yearly total'!B49</f>
         <v>26794</v>
       </c>
       <c r="C49" s="17">
@@ -64932,7 +64932,7 @@
         <v>69</v>
       </c>
       <c r="B50" s="6">
-        <f>'Year total'!B50</f>
+        <f>'Yearly total'!B50</f>
         <v>8498</v>
       </c>
       <c r="C50" s="18">
@@ -65009,7 +65009,7 @@
         <v>70</v>
       </c>
       <c r="B51" s="5">
-        <f>'Year total'!B51</f>
+        <f>'Yearly total'!B51</f>
         <v>21537</v>
       </c>
       <c r="C51" s="17">
@@ -65086,7 +65086,7 @@
         <v>71</v>
       </c>
       <c r="B52" s="6">
-        <f>'Year total'!B52</f>
+        <f>'Yearly total'!B52</f>
         <v>10310</v>
       </c>
       <c r="C52" s="18">
@@ -65163,7 +65163,7 @@
         <v>72</v>
       </c>
       <c r="B53" s="5">
-        <f>'Year total'!B53</f>
+        <f>'Yearly total'!B53</f>
         <v>14087</v>
       </c>
       <c r="C53" s="17">
@@ -65240,7 +65240,7 @@
         <v>73</v>
       </c>
       <c r="B54" s="6">
-        <f>'Year total'!B54</f>
+        <f>'Yearly total'!B54</f>
         <v>7577</v>
       </c>
       <c r="C54" s="18">
@@ -65317,7 +65317,7 @@
         <v>93</v>
       </c>
       <c r="B55" s="11">
-        <f>'Year total'!B55</f>
+        <f>'Yearly total'!B55</f>
         <v>27600</v>
       </c>
       <c r="C55" s="23">
@@ -65394,7 +65394,7 @@
         <v>94</v>
       </c>
       <c r="B56" s="12">
-        <f>'Year total'!B56</f>
+        <f>'Yearly total'!B56</f>
         <v>36104</v>
       </c>
       <c r="C56" s="24">

</xml_diff>